<commit_message>
B1: 2026-04-05 — 131 plays
</commit_message>
<xml_diff>
--- a/daily/2026-04-04.xlsx
+++ b/daily/2026-04-04.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00E0E0E0"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +42,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E1E2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF4444"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0022C55E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F59E0B"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -65,6 +80,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -792,7 +810,6 @@
       <c r="V4" t="n">
         <v>3</v>
       </c>
-      <c r="W4" t="inlineStr"/>
       <c r="X4" t="n">
         <v>2.1</v>
       </c>
@@ -1116,7 +1133,6 @@
       <c r="V8" t="n">
         <v>3</v>
       </c>
-      <c r="W8" t="inlineStr"/>
       <c r="X8" t="n">
         <v>1.3</v>
       </c>
@@ -1686,7 +1702,6 @@
       <c r="V15" t="n">
         <v>9</v>
       </c>
-      <c r="W15" t="inlineStr"/>
       <c r="X15" t="n">
         <v>0</v>
       </c>
@@ -2174,7 +2189,6 @@
       <c r="V21" t="n">
         <v>4</v>
       </c>
-      <c r="W21" t="inlineStr"/>
       <c r="X21" t="n">
         <v>4.8</v>
       </c>
@@ -2580,7 +2594,6 @@
       <c r="V26" t="n">
         <v>4</v>
       </c>
-      <c r="W26" t="inlineStr"/>
       <c r="X26" t="n">
         <v>14</v>
       </c>
@@ -5751,783 +5764,1773 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Jamal Murray</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>24.5</v>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Murray scored 15 pts vs 24.5 line (-9.5), OVER missed by 9.5 pts. Murray played 46 min (+9.4 vs L10 avg of 36.4) — 26% more than expected. Shooting was in line with averages: 46.2% FG (6/13, L10 avg 46.3%). Counter-signals that proved correct: HR L30, HR L10, Defense, FG Trend. Signals that were wrong: Volume, Trend, Context. Projection model targeted 26.5 pts — actual 15 was 11.5 pts off (correct direction). Loss classification: BLOWOUT_EFFECT. Note: Game script invalidated the prop. Consider blowout probability when DEN is involved.</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>BLOWOUT_EFFECT</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Devin Vassell</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="4" t="n">
         <v>12.5</v>
       </c>
+      <c r="E3" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Vassell scored 18 pts vs 12.5 line (+5.5), OVER hit by 5.5 pts. Vassell played 39 min (+9.9 vs L10 avg of 29.3) — 34% more than expected. Shooting was in line with averages: 42.9% FG (6/14, L10 avg 42.0%). Signals that called it correctly: Volume, Context, H2H, Pace, Min Trend (5/10 aligned). Counter-signals that were wrong: HR L30, HR L10, Trend. Projection model targeted 16.7 pts — actual 18 was 1.3 pts close (correct direction). Result classification: MODEL_CORRECT. Note: Projection model accuracy within 2 pts — GBR features are well-calibrated for Vassell in this role.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Dylan Harper</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="4" t="n">
         <v>11.5</v>
       </c>
+      <c r="E4" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Harper scored 12 pts vs 11.5 line (+0.5), OVER hit by 0.5 pts. Harper played 20 min (-3.7 vs L10 avg of 23.9) — 15% less than expected. Shooting efficiency was hot: 71.4% FG (+14.1% vs L10 avg of 57.3%). 5/7 from the field. Signals that called it correctly: Volume, HR L30, HR L10, Trend, Context (8/10 aligned). Counter-signals that were wrong: Defense, H2H. Projection model targeted 13.6 pts — actual 12 was 1.6 pts close (correct direction). Result classification: CLOSE_CALL. Note: Strong signal alignment (8/10) with confirmed result — this player/matchup pattern is reliable for future predictions.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Nikola Jokić</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>LEAN UNDER</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="3" t="n">
         <v>26.5</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Jokić scored 40 pts vs 26.5 line (+13.5), UNDER missed by 13.5 pts. Jokić played 44 min (+8.0 vs L10 avg of 36.0) — 22% more than expected. Shooting was in line with averages: 52.0% FG (13/25, L10 avg 56.7%). Counter-signals that proved correct: Defense, H2H, Pace, FG Trend. Signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 26.3 pts — actual 40 was 13.7 pts off (correct direction). Loss classification: BLOWOUT_EFFECT. Note: Game script invalidated the prop. Consider blowout probability when DEN is involved.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>BLOWOUT_EFFECT</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Tim Hardaway Jr.</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="4" t="n">
         <v>11.5</v>
       </c>
+      <c r="E6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Jr. scored 10 pts vs 11.5 line (-1.5), UNDER hit by 1.5 pts. Minutes were as expected: 26 played vs L10 avg 24.0. Shooting efficiency was hot: 50.0% FG (+10.6% vs L10 avg of 39.4%). 3/6 from the field. Signals that called it correctly: Trend, Defense, H2H, FG Trend, Min Trend (5/10 aligned). Counter-signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 8.3 pts — actual 10 was 1.7 pts close (correct direction). Result classification: CLOSE_CALL. Note: Projection model accuracy within 2 pts — GBR features are well-calibrated for Jr. in this role.</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>De'Aaron Fox</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="3" t="n">
         <v>15.5</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Fox scored 14 pts vs 15.5 line (-1.5), OVER missed by 1.5 pts. Fox played 40 min (+13.2 vs L10 avg of 27.2) — 49% more than expected. Shooting efficiency was cold: 36.8% FG (-12.3% vs L10 avg of 49.1%). 7/19 from the field. Counter-signals that proved correct: HR L30, HR L10, Trend, Defense. Signals that were wrong: Volume, Context, H2H. Projection model targeted 16.5 pts — actual 14 was 2.5 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Victor Wembanyama</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="3" t="n">
         <v>28.5</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Wembanyama scored 34 pts vs 28.5 line (+5.5), UNDER missed by 5.5 pts. Wembanyama played 40 min (+10.5 vs L10 avg of 29.1) — 36% more than expected. Shooting was in line with averages: 47.1% FG (8/17, L10 avg 51.6%). Counter-signals that proved correct: Trend, Defense, H2H, Pace. Signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 27.6 pts — actual 34 was 6.4 pts off (correct direction). Loss classification: MODEL_FAILURE. Note: Model signals were misleading for this matchup — review Wembanyama's recent role and usage for pattern shifts.</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>MODEL_FAILURE</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Keldon Johnson</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="4" t="n">
         <v>12.5</v>
       </c>
+      <c r="E9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Johnson scored 10 pts vs 12.5 line (-2.5), UNDER hit by 2.5 pts. Johnson played 17 min (-6.2 vs L10 avg of 23.6) — 26% less than expected. Shooting efficiency was cold: 30.0% FG (-21.6% vs L10 avg of 51.6%). 3/10 from the field. Signals that called it correctly: Volume, HR L30, Context, H2H (4/10 aligned). Counter-signals that were wrong: HR L10, Trend, Defense. Projection model targeted 10.2 pts — actual 10 was 0.2 pts close (correct direction). Result classification: MODEL_CORRECT. Note: Projection model accuracy within 2 pts — GBR features are well-calibrated for Johnson in this role.</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Christian Braun</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="3" t="n">
         <v>11.5</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Braun scored 21 pts vs 11.5 line (+9.5), UNDER missed by 9.5 pts. Braun played 39 min (+8.7 vs L10 avg of 30.5) — 29% more than expected. Shooting efficiency was cold: 43.8% FG (-15.4% vs L10 avg of 59.2%). 7/16 from the field. Counter-signals that proved correct: Volume, HR L10, Trend, Pace. Signals that were wrong: HR L30, Context, Defense. Projection model targeted 9.0 pts — actual 21 was 12.0 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Stephon Castle</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="3" t="n">
         <v>17.5</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Castle scored 20 pts vs 17.5 line (+2.5), UNDER missed by 2.5 pts. Castle played 40 min (+10.3 vs L10 avg of 30.0) — 34% more than expected. Shooting was in line with averages: 52.9% FG (9/17, L10 avg 48.7%). Counter-signals that proved correct: HR L10, Trend, Pace, Min Trend. Signals that were wrong: Volume, HR L30, Context. Projection model targeted 15.3 pts — actual 20 was 4.7 pts off (correct direction). Loss classification: MODEL_FAILURE. Note: Model signals were misleading for this matchup — review Castle's recent role and usage for pattern shifts.</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>MODEL_FAILURE</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Julian Champagnie</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="4" t="n">
         <v>9.5</v>
       </c>
+      <c r="E12" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Champagnie scored 18 pts vs 9.5 line (+8.5), OVER hit by 8.5 pts. Champagnie played 33 min (+6.4 vs L10 avg of 26.6) — 24% more than expected. Shooting was in line with averages: 50.0% FG (6/12, L10 avg 46.1%). Signals that called it correctly: Volume, HR L30, HR L10, Trend, Context (10/10 aligned). Projection model targeted 13.9 pts — actual 18 was 4.1 pts off (correct direction). Result classification: MODEL_CORRECT. Note: Strong signal alignment (10/10) with confirmed result — this player/matchup pattern is reliable for future predictions.</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Bruce Brown</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="3" t="n">
         <v>6.5</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Brown scored 5 pts vs 6.5 line (-1.5), OVER missed by 1.5 pts. Brown played 11 min (-10.6 vs L10 avg of 21.6) — 49% less than expected. Shooting efficiency was cold: 28.6% FG (-23.9% vs L10 avg of 52.5%). 2/7 from the field. Counter-signals that proved correct: Defense, Min Trend. Signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 8.3 pts — actual 5 was 3.3 pts off (correct direction). Loss classification: MINUTES_SHORTFALL. Note: Minutes were the deciding factor, not scoring rate. Flag Brown for minutes risk in future props if role uncertainty exists.</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>MINUTES_SHORTFALL</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Cameron Johnson</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="4" t="n">
         <v>12.5</v>
       </c>
+      <c r="E14" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Johnson scored 17 pts vs 12.5 line (+4.5), OVER hit by 4.5 pts. Johnson played 39 min (+9.1 vs L10 avg of 30.1) — 30% more than expected. Shooting was in line with averages: 54.5% FG (6/11, L10 avg 51.1%). Signals that called it correctly: HR L10, Trend, Context, H2H, Pace (6/10 aligned). Counter-signals that were wrong: Volume, HR L30, Defense. Projection model targeted 15.3 pts — actual 17 was 1.7 pts close (correct direction). Result classification: MODEL_CORRECT. Note: Projection model accuracy within 2 pts — GBR features are well-calibrated for Johnson in this role.</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Aaron Gordon</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="3" t="n">
         <v>14.5</v>
       </c>
+      <c r="E15" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Gordon scored 15 pts vs 14.5 line (+0.5), UNDER missed by 0.5 pts. Gordon played 41 min (+14.4 vs L10 avg of 26.7) — 54% more than expected. Shooting efficiency was hot: 58.3% FG (+18.3% vs L10 avg of 40.0%). 7/12 from the field. Counter-signals that proved correct: Volume, HR L30, HR L10, H2H. Signals that were wrong: Trend, Context, Defense. Projection model targeted 13.4 pts — actual 15 was 1.6 pts close (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Harrison Barnes</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>SAS @ DEN</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="4" t="n">
         <v>6.5</v>
       </c>
+      <c r="E16" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Barnes scored 8 pts vs 6.5 line (+1.5), OVER hit by 1.5 pts. Barnes played 16 min (-4.9 vs L10 avg of 21.4) — 23% less than expected. Shooting efficiency was hot: 75.0% FG (+25.4% vs L10 avg of 49.6%). 3/4 from the field. Signals that called it correctly: Volume, HR L30, HR L10, Context, Defense (8/10 aligned). Counter-signals that were wrong: Trend, Min Trend. Projection model targeted 11.6 pts — actual 8 was 3.6 pts off (correct direction). Result classification: CLOSE_CALL. Note: Strong signal alignment (8/10) with confirmed result — this player/matchup pattern is reliable for future predictions.</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Kel'el Ware</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>LEAN OVER</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="4" t="n">
         <v>8.5</v>
       </c>
+      <c r="E17" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Ware scored 24 pts vs 8.5 line (+15.5), OVER hit by 15.5 pts. Ware played 36 min (+17.3 vs L10 avg of 18.5) — 94% more than expected. Shooting efficiency was hot: 66.7% FG (+19.6% vs L10 avg of 47.1%). 10/15 from the field. Signals that called it correctly: Volume, HR L30, Context, Defense, H2H (6/10 aligned). Counter-signals that were wrong: HR L10, Trend, FG Trend. Projection model targeted 8.3 pts — actual 24 was 15.7 pts off (wrong direction). Result classification: MODEL_CORRECT. Note: Result confirms Ware's consistency near this line level.</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Alex Sarr</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="5" t="n">
         <v>13.5</v>
       </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Davion Mitchell</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="3" t="n">
         <v>10.5</v>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Mitchell scored 12 pts vs 10.5 line (+1.5), UNDER missed by 1.5 pts. Mitchell played 26 min (-4.9 vs L10 avg of 30.5) — 16% less than expected. Shooting efficiency was hot: 55.6% FG (+7.7% vs L10 avg of 47.9%). 5/9 from the field. Counter-signals that proved correct: HR L10, Trend, Defense, Pace. Signals that were wrong: Volume, HR L30, Context. Projection model targeted 7.9 pts — actual 12 was 4.1 pts off (correct direction). Loss classification: MINUTES_SHORTFALL. Note: Minutes were the deciding factor, not scoring rate. Flag Mitchell for minutes risk in future props if role uncertainty exists.</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>MINUTES_SHORTFALL</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Bilal Coulibaly</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" s="4" t="n">
         <v>12.5</v>
       </c>
+      <c r="E20" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Coulibaly scored 12 pts vs 12.5 line (-0.5), UNDER hit by 0.5 pts. Minutes were as expected: 25 played vs L10 avg 27.3. Shooting efficiency was cold: 38.5% FG (-5.0% vs L10 avg of 43.5%). 5/13 from the field. Signals that called it correctly: Volume, HR L30, Context, H2H, FG Trend (5/10 aligned). Counter-signals that were wrong: HR L10, Trend, Defense. Projection model targeted 9.0 pts — actual 12 was 3.0 pts off (correct direction). Result classification: CLOSE_CALL. Note: Result confirms Coulibaly's consistency near this line level.</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Will Riley</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" s="4" t="n">
         <v>15.5</v>
       </c>
+      <c r="E21" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Riley scored 31 pts vs 15.5 line (+15.5), OVER hit by 15.5 pts. Riley played 37 min (+5.1 vs L10 avg of 31.8) — 16% more than expected. Shooting efficiency was hot: 70.6% FG (+22.3% vs L10 avg of 48.3%). 12/17 from the field. Signals that called it correctly: HR L10, Trend, Context, Defense, Pace (7/10 aligned). Counter-signals that were wrong: Volume, HR L30, H2H. Projection model targeted 19.4 pts — actual 31 was 11.6 pts off (correct direction). Result classification: MODEL_CORRECT. Note: Result confirms Riley's consistency near this line level.</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Pelle Larsson</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="4" t="n">
         <v>15.5</v>
       </c>
+      <c r="E22" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Larsson scored 16 pts vs 15.5 line (+0.5), OVER hit by 0.5 pts. Larsson played 24 min (-8.2 vs L10 avg of 32.0) — 26% less than expected. Shooting efficiency was hot: 60.0% FG (+8.2% vs L10 avg of 51.8%). 6/10 from the field. Signals that called it correctly: Trend, Defense, Pace, FG Trend, Min Trend (5/10 aligned). Counter-signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 17.0 pts — actual 16 was 1.0 pts close (correct direction). Result classification: CLOSE_CALL. Note: Projection model accuracy within 2 pts — GBR features are well-calibrated for Larsson in this role.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Tyler Herro</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="5" t="n">
         <v>24.5</v>
       </c>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="inlineStr"/>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Jaime Jaquez Jr.</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="3" t="n">
         <v>16.5</v>
       </c>
+      <c r="E24" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Jr. scored 32 pts vs 16.5 line (+15.5), UNDER missed by 15.5 pts. Jr. played 32 min (+6.3 vs L10 avg of 25.7) — 25% more than expected. Shooting efficiency was hot: 66.7% FG (+20.6% vs L10 avg of 46.1%). 12/18 from the field. Counter-signals that proved correct: Trend, Defense, Pace. Signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 15.0 pts — actual 32 was 17.0 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Andrew Wiggins</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" s="3" t="n">
         <v>15.5</v>
       </c>
+      <c r="E25" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Wiggins scored 21 pts vs 15.5 line (+5.5), UNDER missed by 5.5 pts. Minutes were as expected: 26 played vs L10 avg 28.5. Shooting efficiency was hot: 63.6% FG (+13.9% vs L10 avg of 49.7%). 7/11 from the field. Counter-signals that proved correct: Defense, H2H, Pace, FG Trend. Signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 11.0 pts — actual 21 was 10.0 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Tre Johnson</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D26" s="3" t="n">
         <v>12.5</v>
       </c>
+      <c r="E26" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Johnson scored 11 pts vs 12.5 line (-1.5), OVER missed by 1.5 pts. Minutes were as expected: 25 played vs L10 avg 23.2. Shooting was in line with averages: 38.5% FG (5/13, L10 avg 37.1%). Counter-signals that proved correct: Volume, HR L30, HR L10, Trend. Signals that were wrong: Context, Defense, Pace. Projection model targeted 14.4 pts — actual 11 was 3.4 pts off (correct direction). Loss classification: CLOSE_CALL. Note: Within 2 pts — direction was sound. Small execution variance, no model adjustment needed.</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Bam Adebayo</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>WAS @ MIA</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="3" t="n">
         <v>24.5</v>
       </c>
+      <c r="E27" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Adebayo scored 14 pts vs 24.5 line (-10.5), OVER missed by 10.5 pts. Adebayo played 24 min (-12.0 vs L10 avg of 36.2) — 33% less than expected. Shooting efficiency was hot: 50.0% FG (+11.3% vs L10 avg of 38.7%). 3/6 from the field. Counter-signals that proved correct: Volume, HR L30, HR L10, Trend. Signals that were wrong: Defense, H2H, Pace. Projection model targeted 30.3 pts — actual 14 was 16.3 pts off (correct direction). Loss classification: MINUTES_SHORTFALL. Note: Minutes were the deciding factor, not scoring rate. Flag Adebayo for minutes risk in future props if role uncertainty exists.</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>MINUTES_SHORTFALL</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Kelly Oubre Jr.</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="4" t="n">
         <v>15.5</v>
       </c>
+      <c r="E28" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Jr. scored 3 pts vs 15.5 line (-12.5), UNDER hit by 12.5 pts. Jr. played 24 min (-5.1 vs L10 avg of 29.4) — 17% less than expected. Shooting efficiency was cold: 25.0% FG (-23.1% vs L10 avg of 48.1%). 1/4 from the field. Signals that called it correctly: Volume, HR L30, HR L10, Context, Defense (8/10 aligned). Counter-signals that were wrong: Trend, FG Trend. Projection model targeted 10.1 pts — actual 3 was 7.1 pts off (correct direction). Result classification: MODEL_CORRECT. Note: Strong signal alignment (8/10) with confirmed result — this player/matchup pattern is reliable for future predictions.</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Duncan Robinson</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="3" t="n">
         <v>12.5</v>
       </c>
+      <c r="E29" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Robinson scored 11 pts vs 12.5 line (-1.5), OVER missed by 1.5 pts. Robinson played 23 min (-3.8 vs L10 avg of 27.2) — 14% less than expected. Shooting efficiency was hot: 57.1% FG (+11.6% vs L10 avg of 45.5%). 4/7 from the field. Counter-signals that proved correct: Volume, HR L10, Pace, FG Trend. Signals that were wrong: HR L30, Trend, Context. Projection model targeted 13.3 pts — actual 11 was 2.3 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Daniss Jenkins</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" s="4" t="n">
         <v>16.5</v>
       </c>
+      <c r="E30" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Jenkins scored 16 pts vs 16.5 line (-0.5), UNDER hit by 0.5 pts. Jenkins played 32 min (-3.2 vs L10 avg of 34.7) — 9% less than expected. Shooting efficiency was cold: 36.4% FG (-9.6% vs L10 avg of 46.0%). 4/11 from the field. Signals that called it correctly: Volume, HR L30, Context, H2H, Pace (5/10 aligned). Counter-signals that were wrong: HR L10, Trend, Defense. Projection model targeted 12.9 pts — actual 16 was 3.1 pts off (correct direction). Result classification: CLOSE_CALL. Note: Result confirms Jenkins's consistency near this line level.</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>VJ Edgecombe</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="3" t="n">
         <v>16.5</v>
       </c>
+      <c r="E31" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Edgecombe scored 19 pts vs 16.5 line (+2.5), UNDER missed by 2.5 pts. Minutes were as expected: 35 played vs L10 avg 33.5. Shooting efficiency was cold: 38.9% FG (-13.2% vs L10 avg of 52.1%). 7/18 from the field. Counter-signals that proved correct: Volume, HR L10, FG Trend, Min Trend. Signals that were wrong: HR L30, Trend, Context. Projection model targeted 11.1 pts — actual 19 was 7.9 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Kevin Huerter</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>LEAN OVER</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="3" t="n">
         <v>9.5</v>
       </c>
+      <c r="E32" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Huerter scored 5 pts vs 9.5 line (-4.5), OVER missed by 4.5 pts. Minutes were as expected: 25 played vs L10 avg 23.6. Shooting efficiency was cold: 22.2% FG (-24.8% vs L10 avg of 47.0%). 2/9 from the field. Counter-signals that proved correct: Volume, HR L30, HR L10, Context. Signals that were wrong: Trend, Defense, H2H. Projection model targeted 9.6 pts — actual 5 was 4.6 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Dominick Barlow</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="4" t="n">
         <v>8.5</v>
       </c>
+      <c r="E33" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Barlow scored 8 pts vs 8.5 line (-0.5), UNDER hit by 0.5 pts. Barlow played 29 min (+7.7 vs L10 avg of 21.3) — 36% more than expected. Shooting efficiency was cold: 50.0% FG (-9.9% vs L10 avg of 59.9%). 3/6 from the field. Signals that called it correctly: Volume, HR L30, HR L10, Trend, Context (9/10 aligned). Counter-signals that were wrong: FG Trend. Projection model targeted 7.3 pts — actual 8 was 0.7 pts close (correct direction). Result classification: CLOSE_CALL. Note: Strong signal alignment (9/10) with confirmed result — this player/matchup pattern is reliable for future predictions.</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>CLOSE_CALL</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Tobias Harris</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D34" s="3" t="n">
         <v>13.5</v>
       </c>
+      <c r="E34" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Harris scored 19 pts vs 13.5 line (+5.5), UNDER missed by 5.5 pts. Minutes were as expected: 27 played vs L10 avg 26.7. Shooting was in line with averages: 53.8% FG (7/13, L10 avg 54.9%). Counter-signals that proved correct: Trend, Defense, H2H, FG Trend. Signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 12.1 pts — actual 19 was 6.9 pts off (correct direction). Loss classification: MODEL_FAILURE. Note: Model signals were misleading for this matchup — review Harris's recent role and usage for pattern shifts.</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>MODEL_FAILURE</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Jalen Duren</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" s="4" t="n">
         <v>22.5</v>
       </c>
+      <c r="E35" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Duren scored 16 pts vs 22.5 line (-6.5), UNDER hit by 6.5 pts. Minutes were as expected: 30 played vs L10 avg 32.0. Shooting efficiency was cold: 62.5% FG (-5.3% vs L10 avg of 67.8%). 5/8 from the field. Signals that called it correctly: Volume, Context, H2H, Pace (4/10 aligned). Counter-signals that were wrong: HR L30, HR L10, Trend. Projection model targeted 18.6 pts — actual 16 was 2.6 pts off (correct direction). Result classification: MODEL_CORRECT. Note: Result confirms Duren's consistency near this line level.</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Tyrese Maxey</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D36" s="4" t="n">
         <v>28.5</v>
       </c>
+      <c r="E36" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Maxey scored 23 pts vs 28.5 line (-5.5), UNDER hit by 5.5 pts. Maxey played 33 min (-4.0 vs L10 avg of 37.2) — 11% less than expected. Shooting was in line with averages: 47.1% FG (8/17, L10 avg 45.3%). Signals that called it correctly: Volume, HR L30, HR L10, Trend, Context (7/10 aligned). Counter-signals that were wrong: H2H, FG Trend, Min Trend. Projection model targeted 27.2 pts — actual 23 was 4.2 pts off (correct direction). Result classification: MODEL_CORRECT. Note: Result confirms Maxey's consistency near this line level.</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Quentin Grimes</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D37" s="4" t="n">
         <v>12.5</v>
       </c>
+      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Grimes scored 0 pts vs 12.5 line (-12.5), UNDER hit by 12.5 pts. Grimes played 17 min (-13.3 vs L10 avg of 30.7) — 43% less than expected. Shooting efficiency was cold: 0.0% FG (-50.0% vs L10 avg of 50.0%). 0/4 from the field. Signals that called it correctly: Trend, Defense, H2H, Pace (4/10 aligned). Counter-signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 9.2 pts — actual 0 was 9.2 pts off (correct direction). Result classification: MODEL_CORRECT. Note: Result confirms Grimes's consistency near this line level.</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Ausar Thompson</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>LEAN UNDER</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D38" s="3" t="n">
         <v>9.5</v>
       </c>
+      <c r="E38" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Thompson scored 14 pts vs 9.5 line (+4.5), UNDER missed by 4.5 pts. Thompson played 25 min (-3.7 vs L10 avg of 28.5) — 13% less than expected. Shooting efficiency was hot: 63.6% FG (+10.8% vs L10 avg of 52.8%). 7/11 from the field. Counter-signals that proved correct: Defense, H2H, FG Trend, Min Trend. Signals that were wrong: Volume, HR L30, HR L10. Projection model targeted 9.6 pts — actual 14 was 4.4 pts off (wrong direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Paul Reed</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" s="4" t="n">
         <v>7.5</v>
       </c>
+      <c r="E39" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>WIN — Reed scored 10 pts vs 7.5 line (+2.5), OVER hit by 2.5 pts. Minutes were as expected: 18 played vs L10 avg 17.8. Shooting efficiency was hot: 80.0% FG (+16.2% vs L10 avg of 63.8%). 4/5 from the field. Signals that called it correctly: Volume, HR L30, HR L10, Trend, Context (8/10 aligned). Counter-signals that were wrong: H2H, Pace. Projection model targeted 7.9 pts — actual 10 was 2.1 pts off (correct direction). Result classification: MODEL_CORRECT. Note: Strong signal alignment (8/10) with confirmed result — this player/matchup pattern is reliable for future predictions.</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>MODEL_CORRECT</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>Adem Bona</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>DET @ PHI</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>UNDER</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D40" s="3" t="n">
         <v>6.5</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>LOSS — Bona scored 10 pts vs 6.5 line (+3.5), UNDER missed by 3.5 pts. Bona played 23 min (+6.8 vs L10 avg of 16.3) — 42% more than expected. Shooting efficiency was hot: 100.0% FG (+43.8% vs L10 avg of 56.2%). 5/5 from the field. All 10 agreeing signals (Volume, HR L30, HR L10, Trend) were wrong — result went directly against the consensus. Projection model targeted 2.5 pts — actual 10 was 7.5 pts off (correct direction). Loss classification: SHOOTING_VARIANCE. Note: Volume and opportunity signals were correct but shooting efficiency diverged. Normal variance — per-minute output was on track.</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>SHOOTING_VARIANCE</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05 07:40</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>